<commit_message>
Add user stories and acceptance criteria for article formatting and search bar functionality
- Created detailed user stories for site editors to enhance article formatting control, including acceptance criteria and test outlines.
- Implemented user stories for website visitors regarding the search bar placement and functionality, ensuring accessibility and usability.
- Included metrics and diversity scores for each user story to evaluate effectiveness and user satisfaction.
- Updated email list for project stakeholders.
</commit_message>
<xml_diff>
--- a/data/user_story_submit_example.xlsx
+++ b/data/user_story_submit_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carrie0925/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carrie0925/Desktop/NTHU/0.thesis/Dspy Implement/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A275386-385F-B44A-BFDE-30BD94AD01D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357D3815-B89E-404D-9FEC-5C37847CC098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,20 +22,21 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>description</t>
-  </si>
-  <si>
     <t>As a site editor, I want to have pretty good control over how the article, so that articles are visually appealing.</t>
   </si>
   <si>
     <t>I want a search bar on the top of the page.</t>
   </si>
+  <si>
+    <t>description(You can delete examples and add maximum 5 user stories)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -53,6 +54,13 @@
       <name val="Arial"/>
       <family val="3"/>
       <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -76,9 +84,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -301,18 +310,18 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>